<commit_message>
feat: Add and enhance animated loading screen
</commit_message>
<xml_diff>
--- a/data/attendance/attendance.xlsx
+++ b/data/attendance/attendance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,168 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>18:13:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>31715255</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Michael Jackson</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>22:36:05</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>31715256</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Amiyah Mosley</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>22:36:11</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>31715255</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Michael Jackson</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>